<commit_message>
Evlaución estricta con formatao de json y md segun isntrucciones desde ficheros de configuración. Ademñas, las rúbicas se cargan en función de la tipología del TFM derivada de la lectura de etiqueta asociado al documento del TFE aportado por el alumno.
</commit_message>
<xml_diff>
--- a/automatedEval/TFM_Evaluator_Prompt_Package/rubrica MUDPE.xlsx
+++ b/automatedEval/TFM_Evaluator_Prompt_Package/rubrica MUDPE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanjo/Documents/Personal/JJVR/automatizaciones/automatedEval/TFM_Evaluator_Prompt_Package/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF928049-656B-DC45-99A3-3C4217C0A86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B1C3F0-F90F-6D41-912C-96C6CE896BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="21460" yWindow="500" windowWidth="26800" windowHeight="28260" xr2:uid="{22A2D1EC-3F8C-434E-B6E5-5DB57C6AFD5E}"/>
   </bookViews>
@@ -387,10 +387,10 @@
     </r>
     <r>
       <rPr>
-        <sz val="12"/>
+        <sz val="14"/>
         <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <rFont val="Aptos Display"/>
+        <scheme val="major"/>
       </rPr>
       <t>Estilo formal/académico</t>
     </r>
@@ -403,10 +403,10 @@
     </r>
     <r>
       <rPr>
-        <sz val="12"/>
+        <sz val="14"/>
         <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <rFont val="Aptos Display"/>
+        <scheme val="major"/>
       </rPr>
       <t>· Portada; Resumen; Índice
 · Introducción; Justificación; objetivos
@@ -420,7 +420,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -448,22 +448,35 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Aptos Display"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="5">
@@ -603,61 +616,62 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -994,266 +1008,266 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AA496D9-71D8-0343-844B-38BFC7DE0A68}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.1640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="40.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="46.33203125" style="1" customWidth="1"/>
     <col min="6" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="340">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:6" ht="209" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="5"/>
-    </row>
-    <row r="3" spans="1:6" ht="409.6">
-      <c r="A3" s="6" t="s">
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="171" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="5"/>
-    </row>
-    <row r="4" spans="1:6" ht="289">
-      <c r="A4" s="9" t="s">
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" ht="190" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:6" ht="323">
-      <c r="A5" s="10" t="s">
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" ht="190" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="6" spans="1:6" ht="409.6">
-      <c r="A6" s="9" t="s">
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="7" spans="1:6" ht="204">
-      <c r="A7" s="9" t="s">
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" ht="171" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="8" spans="1:6" ht="187">
-      <c r="A8" s="9" t="s">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" ht="133" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="5"/>
-    </row>
-    <row r="9" spans="1:6" ht="153">
-      <c r="A9" s="9" t="s">
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" ht="95" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="5"/>
-    </row>
-    <row r="10" spans="1:6" ht="221">
-      <c r="A10" s="9" t="s">
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" ht="133" x14ac:dyDescent="0.2">
+      <c r="A10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="5"/>
-    </row>
-    <row r="11" spans="1:6" ht="255">
-      <c r="A11" s="14" t="s">
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" ht="152" x14ac:dyDescent="0.2">
+      <c r="A11" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="12" spans="1:6" ht="204">
-      <c r="A12" s="14" t="s">
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" ht="133" x14ac:dyDescent="0.2">
+      <c r="A12" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="1:6" ht="388">
-      <c r="A13" s="14" t="s">
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" ht="209" x14ac:dyDescent="0.2">
+      <c r="A13" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:6" ht="273" thickBot="1">
-      <c r="A14" s="15" t="s">
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" ht="153" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="F14" s="18"/>
+      <c r="F14" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
chore(release): finalizar archivado UNIR_Grading y sincronizar movimientos
</commit_message>
<xml_diff>
--- a/automatedEval/TFM_Evaluator_Prompt_Package/rubrica MUDPE.xlsx
+++ b/automatedEval/TFM_Evaluator_Prompt_Package/rubrica MUDPE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanjo/Documents/Personal/JJVR/automatizaciones/automatedEval/TFM_Evaluator_Prompt_Package/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B1C3F0-F90F-6D41-912C-96C6CE896BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2BB7A0-F5A9-4141-B5C3-3D656828B992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="21460" yWindow="500" windowWidth="26800" windowHeight="28260" xr2:uid="{22A2D1EC-3F8C-434E-B6E5-5DB57C6AFD5E}"/>
   </bookViews>
@@ -365,18 +365,6 @@
 · Utiliza gestos para enfatizar los contenidos importantes, domina la comunicación no verbal.</t>
   </si>
   <si>
-    <t>Nivel 4</t>
-  </si>
-  <si>
-    <t>Nivel 1</t>
-  </si>
-  <si>
-    <t>Nivel 2</t>
-  </si>
-  <si>
-    <t>Nivel 3</t>
-  </si>
-  <si>
     <t>Criterio</t>
   </si>
   <si>
@@ -415,12 +403,24 @@
 · Limitaciones, principales amenazas y alternativas                                                                                                                                                                                                                                                                                                                           · Referencias bibliográficas</t>
     </r>
   </si>
+  <si>
+    <t>Nivel 1  (0-4)</t>
+  </si>
+  <si>
+    <t>Nivel 2 (5-6)</t>
+  </si>
+  <si>
+    <t>Nivel 3 (7-8)</t>
+  </si>
+  <si>
+    <t>Nivel 4 (9-10)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -478,8 +478,23 @@
       <name val="Aptos Display"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,6 +519,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -613,10 +634,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -673,8 +695,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="60% - Énfasis1" xfId="1" builtinId="32"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1020,24 +1045,24 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>63</v>
+      <c r="D1" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="209" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>0</v>
@@ -1055,7 +1080,7 @@
     </row>
     <row r="3" spans="1:6" ht="171" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>4</v>

</xml_diff>